<commit_message>
Modified the logic of mapping the user password hash
</commit_message>
<xml_diff>
--- a/migrated_backend/storage/RechiCMS.xlsx
+++ b/migrated_backend/storage/RechiCMS.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="users" sheetId="1" state="visible" r:id="rId1"/>
@@ -23,16 +22,29 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy/m/d h:mm"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -43,7 +55,14 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
     <border>
       <left/>
       <right/>
@@ -53,14 +72,35 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf numFmtId="3" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -139,10 +179,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:sysClr lastClr="000000" val="windowText"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:sysClr lastClr="FFFFFF" val="window"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="1F497D"/>
@@ -180,69 +220,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Times New Roman" script="Arab"/>
+        <a:font typeface="Times New Roman" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="MoolBoran" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Times New Roman" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
+        <a:font typeface="맑은 고딕" script="Hang"/>
+        <a:font typeface="宋体" script="Hans"/>
+        <a:font typeface="新細明體" script="Hant"/>
+        <a:font typeface="Arial" script="Arab"/>
+        <a:font typeface="Arial" script="Hebr"/>
+        <a:font typeface="Tahoma" script="Thai"/>
+        <a:font typeface="Nyala" script="Ethi"/>
+        <a:font typeface="Vrinda" script="Beng"/>
+        <a:font typeface="Shruti" script="Gujr"/>
+        <a:font typeface="DaunPenh" script="Khmr"/>
+        <a:font typeface="Tunga" script="Knda"/>
+        <a:font typeface="Raavi" script="Guru"/>
+        <a:font typeface="Euphemia" script="Cans"/>
+        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
+        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
+        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
+        <a:font typeface="MV Boli" script="Thaa"/>
+        <a:font typeface="Mangal" script="Deva"/>
+        <a:font typeface="Gautami" script="Telu"/>
+        <a:font typeface="Latha" script="Taml"/>
+        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
+        <a:font typeface="Kalinga" script="Orya"/>
+        <a:font typeface="Kartika" script="Mlym"/>
+        <a:font typeface="DokChampa" script="Laoo"/>
+        <a:font typeface="Iskoola Pota" script="Sinh"/>
+        <a:font typeface="Mongolian Baiti" script="Mong"/>
+        <a:font typeface="Arial" script="Viet"/>
+        <a:font typeface="Microsoft Uighur" script="Uigh"/>
+        <a:font typeface="Sylfaen" script="Geor"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -266,54 +308,53 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:tint val="15000"/>
                 <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="1"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:shade val="51000"/>
+                <a:tint val="51000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="80000">
               <a:schemeClr val="phClr">
-                <a:shade val="93000"/>
+                <a:tint val="15000"/>
                 <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="94000"/>
+                <a:tint val="94000"/>
                 <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="16200000" scaled="0"/>
+          <a:lin scaled="1" ang="16200000"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
           <a:solidFill>
             <a:schemeClr val="phClr">
-              <a:shade val="95000"/>
+              <a:shade val="9500"/>
               <a:satMod val="105000"/>
             </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -323,7 +364,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -332,7 +373,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -341,7 +382,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -349,10 +390,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot lat="0" lon="0" rev="0"/>
+              <a:rot rev="0" lon="0" lat="0"/>
             </a:camera>
-            <a:lightRig rig="threePt" dir="t">
-              <a:rot lat="0" lon="0" rev="1200000"/>
+            <a:lightRig dir="t" rig="threePt">
+              <a:rot rev="1200000" lon="0" lat="0"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -381,7 +422,7 @@
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="20000"/>
+                <a:tint val="20000"/>
                 <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
@@ -394,13 +435,12 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="80000"/>
                 <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="30000"/>
+                <a:tint val="80000"/>
                 <a:satMod val="200000"/>
               </a:schemeClr>
             </a:gs>
@@ -420,856 +460,997 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="4" max="4"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="5" max="5"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="6" max="6"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="7" max="7"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="8" max="8"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>username</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>password</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>role</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>is_active</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="19.5" customHeight="1">
+      <c r="A2" s="6" t="n"/>
+      <c r="B2" s="6" t="n"/>
+      <c r="C2" s="6" t="n"/>
+      <c r="D2" s="6" t="n"/>
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="6" t="n"/>
+      <c r="G2" s="7" t="n"/>
+      <c r="H2" s="7" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Rechi_Cons</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>rechiconstruction@yahoo.in</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>$2b$12$rRySr4E1IjGhUuIi1Ei5LuEllnF7e6uCgYtdxSUAiQmGijrTofILy</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>$2b$12$xKeTv7EQg0Nfdb6REbMrM.H50/hRrL1Gwa8AEhBMheKcoDN/Phewy</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
         <is>
           <t>admin</t>
         </is>
       </c>
-      <c r="F2" t="b">
+      <c r="F3" t="b">
         <v>1</v>
       </c>
-      <c r="G2" s="1" t="n">
-        <v>46243.93026865477</v>
-      </c>
-      <c r="H2" s="1" t="n">
-        <v>46243.93026865533</v>
+      <c r="G3" s="8" t="n">
+        <v>46252.92288191905</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>46252.92288191969</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="4" max="4"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="5" max="5"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="6" max="6"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="7" max="7"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="8" max="8"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="9" max="9"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="10" max="10"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="11" max="11"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="12" max="12"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="13" max="13"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="14" max="14"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="15" max="15"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="16" max="16"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="17" max="17"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>company_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>about</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>mission</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>vision</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>alternate_phone</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>address</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>facebook</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>instagram</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>youtube</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>logo</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>favicon</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="6" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="18.75" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Rechi Cons</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Leading construction company.</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Deliver quality.</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Trusted Builder.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>9999999999</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>8888888888</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="F2" s="3" t="n">
+        <v>9999999999</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>8888888888</v>
+      </c>
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>info@rechi.com</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>West Bengal</t>
         </is>
       </c>
-      <c r="P2" s="1" t="n">
-        <v>46238.80708146991</v>
-      </c>
-      <c r="Q2" s="1" t="n">
-        <v>46238.81447127314</v>
+      <c r="J2" s="6" t="n"/>
+      <c r="K2" s="6" t="n"/>
+      <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="n"/>
+      <c r="N2" s="6" t="n"/>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="4" t="inlineStr">
+        <is>
+          <t>Wed Aug 05 2026 00:52:11 GMT+0530 (India Standard Time)</t>
+        </is>
+      </c>
+      <c r="Q2" s="4" t="inlineStr">
+        <is>
+          <t>Wed Aug 05 2026 01:02:50 GMT+0530 (India Standard Time)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="4" max="4"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="5" max="5"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="6" max="6"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="7" max="7"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>display_order</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>is_active</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
+      <c r="F1" s="6" t="n"/>
+      <c r="G1" s="6" t="n"/>
+    </row>
+    <row r="2" ht="18.75" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>completed_projects</t>
         </is>
       </c>
-      <c r="D2" t="n">
+      <c r="D2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E2" t="b">
-        <v>1</v>
-      </c>
-      <c r="F2" s="1" t="n">
-        <v>46238.82961914352</v>
-      </c>
-      <c r="G2" s="1" t="n">
-        <v>46238.82961914352</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="n">
+      <c r="E2" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Wed Aug 05 2026 01:24:39 GMT+0530 (India Standard Time)</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Wed Aug 05 2026 01:24:39 GMT+0530 (India Standard Time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18.75" customHeight="1">
+      <c r="A3" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="6" t="inlineStr">
         <is>
           <t>Ongoing</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>ongoing_projects</t>
         </is>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E3" t="b">
-        <v>1</v>
-      </c>
-      <c r="F3" s="1" t="n">
-        <v>46238.83038510416</v>
-      </c>
-      <c r="G3" s="1" t="n">
-        <v>46238.83038510416</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="n">
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>Wed Aug 05 2026 01:25:45 GMT+0530 (India Standard Time)</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>Wed Aug 05 2026 01:25:45 GMT+0530 (India Standard Time)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18.75" customHeight="1">
+      <c r="A4" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Upcoming</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>upcoming_projects</t>
         </is>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="E4" t="b">
-        <v>1</v>
-      </c>
-      <c r="F4" s="1" t="n">
-        <v>46238.8308353125</v>
-      </c>
-      <c r="G4" s="1" t="n">
-        <v>46238.8308353125</v>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>Wed Aug 05 2026 01:26:24 GMT+0530 (India Standard Time)</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>Wed Aug 05 2026 01:26:24 GMT+0530 (India Standard Time)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="2" max="2"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="4" max="4"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="5" max="5"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="6" max="6"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="7" max="7"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="8" max="8"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="9" max="9"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="10" max="10"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="11" max="11"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="12" max="12"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="13" max="13"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="14" max="14"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="15" max="15"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="16" max="16"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>category_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>short_description</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>location</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>builder</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>status</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>rera_number</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>thumbnail</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>is_featured</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="5" t="inlineStr">
         <is>
           <t>display_order</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="18.75" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Anandi Apartments</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>anandi-apartments</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Apartment build on strong base with adequate spacing.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Lambda Beta string case object trust</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Kolkata</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Rechi Constructions</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I2" s="6" t="inlineStr">
         <is>
           <t>Completed</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J2" s="6" t="inlineStr">
         <is>
           <t>NULL</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="6" t="inlineStr">
         <is>
           <t>RS0001</t>
         </is>
       </c>
-      <c r="M2" t="b">
+      <c r="L2" s="6" t="n"/>
+      <c r="M2" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="N2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O2" s="1" t="n">
-        <v>46240.91079559028</v>
-      </c>
-      <c r="P2" s="1" t="n">
-        <v>46240.9121571412</v>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>Fri Aug 07 2026 03:21:32 GMT+0530 (India Standard Time)</t>
+        </is>
+      </c>
+      <c r="P2" s="4" t="inlineStr">
+        <is>
+          <t>Fri Aug 07 2026 03:23:30 GMT+0530 (India Standard Time)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="2" max="2"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="4" max="4"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>project_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>image_path</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>image_type</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="18.75" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>projects/gallery/7ca370c786d349979d085eeff30c9385.png</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>gallery</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
+    <row r="3" ht="18.75" customHeight="1">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>projects/gallery/3cbdf8595bec43f9bcf4285427f41827.png</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>gallery</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
+    <row r="4" ht="18.75" customHeight="1">
+      <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>projects/floorplans/2c709928df2f47e49e67c412fad4ea54.png</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>floorplan</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
+    <row r="5" ht="18.75" customHeight="1">
+      <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>projects/siteplans/8a42d57b41a94705a46246dbbb41a745.png</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>siteplan</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>project_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="4" max="4"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="5" max="5"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="6" max="6"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="7" max="7"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="8" max="8"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="9" max="9"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>slug</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>content</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>image_path</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>display_order</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>is_active</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>updated_at</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="18.75" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>stringggggg</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>stringggggg</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>strinnnnng</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="E2" s="6" t="n"/>
+      <c r="F2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="G2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" s="1" t="n">
-        <v>46240.8597131713</v>
-      </c>
-      <c r="I2" s="1" t="n">
-        <v>46240.86808270833</v>
+      <c r="G2" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Fri Aug 07 2026 02:07:59 GMT+0530 (India Standard Time)</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Fri Aug 07 2026 02:20:02 GMT+0530 (India Standard Time)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="3" max="3"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="4" max="4"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="5" max="5"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="6" max="6"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="7" max="7"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="8" max="8"/>
+    <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="9" max="9"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="18.75" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>subject</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>message</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>project_id</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>is_read</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>created_at</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="n">
+    <row r="2" ht="18.75" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>sting kumar</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>sting@kumar.com</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>9900887766</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="D2" s="3" t="n">
+        <v>9900887766</v>
+      </c>
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Conversation about anandi villa.</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>wiufbwb iwbvwba yuawvebv uywvw  nsmcama c iub a, iacaba qibfww bwcuwcw</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="G2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H2" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="1" t="n">
-        <v>46243.91443983796</v>
+      <c r="H2" s="6" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Mon Aug 10 2026 03:26:47 GMT+0530 (India Standard Time)</t>
+        </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated payload for other services
</commit_message>
<xml_diff>
--- a/migrated_backend/storage/RechiCMS.xlsx
+++ b/migrated_backend/storage/RechiCMS.xlsx
@@ -464,7 +464,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
@@ -556,10 +556,10 @@
         <v>1</v>
       </c>
       <c r="G3" s="8" t="n">
-        <v>46252.92288191905</v>
+        <v>46252.92288192129</v>
       </c>
       <c r="H3" s="8" t="n">
-        <v>46252.92288191969</v>
+        <v>46252.92288192129</v>
       </c>
     </row>
   </sheetData>
@@ -574,7 +574,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
@@ -751,7 +751,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
@@ -902,7 +902,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="2" max="2"/>
@@ -1088,7 +1088,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="2" max="2"/>
@@ -1202,7 +1202,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
@@ -1237,8 +1237,8 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>
@@ -1299,42 +1299,67 @@
       </c>
     </row>
     <row r="2" ht="18.75" customHeight="1">
-      <c r="A2" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="6" t="inlineStr">
-        <is>
-          <t>stringggggg</t>
-        </is>
-      </c>
-      <c r="C2" s="6" t="inlineStr">
-        <is>
-          <t>stringggggg</t>
-        </is>
-      </c>
-      <c r="D2" s="6" t="inlineStr">
-        <is>
-          <t>strinnnnng</t>
-        </is>
-      </c>
-      <c r="E2" s="6" t="n"/>
-      <c r="F2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>Fri Aug 07 2026 02:07:59 GMT+0530 (India Standard Time)</t>
-        </is>
-      </c>
-      <c r="I2" s="4" t="inlineStr">
-        <is>
-          <t>Fri Aug 07 2026 02:20:02 GMT+0530 (India Standard Time)</t>
-        </is>
+      <c r="A2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Interior Designing and Execution</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>interior-designing-and-execution</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>[{"type": "paragraph", "text": "Rechi Construction provides end-to-end solutions in terms of purchase of completed furnished flats. It has a strong liaison with designers, carpenters, decorators, etc. and can execute projects at a fraction of the cost of other solution providers.", "items": null}, {"type": "bullet_list", "text": null, "items": ["Assistance in mutation of names", "Assistance in transfer and sale of properties", "Assistance in legal matters related to land and property", "Assistance in Home Loan sanctioning"]}]</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>1</v>
+      </c>
+      <c r="G2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H2" s="8" t="n">
+        <v>46265.45483527778</v>
+      </c>
+      <c r="I2" s="8" t="n">
+        <v>46265.45483527778</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Property Consultation</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>property-consultation</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>[{"type": "paragraph", "text": "Rechi Construction provides professional assistance throughout the property consultation and planning process.", "items": null}, {"type": "bullet_list", "text": null, "items": ["Property selection and consultation", "Assistance with property documentation", "Site visits and evaluation", "Project planning and execution guidance"]}]</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G3" t="b">
+        <v>1</v>
+      </c>
+      <c r="H3" s="8" t="n">
+        <v>46265.46769271186</v>
+      </c>
+      <c r="I3" s="8" t="n">
+        <v>46265.46769271192</v>
       </c>
     </row>
   </sheetData>
@@ -1349,7 +1374,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="5" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="6" min="2" max="2"/>

</xml_diff>

<commit_message>
Updated project data in the excel file
</commit_message>
<xml_diff>
--- a/migrated_backend/storage/RechiCMS.xlsx
+++ b/migrated_backend/storage/RechiCMS.xlsx
@@ -1041,74 +1041,70 @@
       </c>
     </row>
     <row r="2" ht="19.5" customHeight="1">
-      <c r="A2" s="7" t="n">
-        <v>2</v>
-      </c>
-      <c r="B2" s="7" t="n">
+      <c r="A2" t="n">
         <v>3</v>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="inlineStr">
         <is>
           <t>ANANDI VISTA</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>anandi-vista</t>
         </is>
       </c>
-      <c r="E2" s="8" t="n"/>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>[{"type": "paragraph", "text": "Taking advantage of the features of the Complex, the three bedrooms with two bathrooms and a huge living room with kitchen and dining room were created, thus making the space much brighter, more spacious and most good things are its the sided open."}, {"type": "paragraph", "text": "The kitchen is fully open space concept, several storage options."}, {"type": "paragraph", "text": "The bathrooms have high-quality sanitary ware and best design tiles to match the style of the apartment."}, {"type": "paragraph", "text": "The living room has a high-quality spacious."}, {"type": "paragraph", "text": "ANANDI VISTA - Sensibility that is entrenched in the creation, the entire project is a marvel that consists of features and facilities that make life easy and comfortable. The project is beautifully structured with innovative designs and elegant structures that form neat layouts for your dream home. The retreat serves with all up to date services and modern outlay which drives you to a world of calm and peace. The designs and the features are contemporary with supreme class that has an upper hand in its furnishing. The interior and the exteriors of the project are intended with user friendliness and simple living yet high in style for an ease life. The location and the ambiance have a lush green world around you with an elegant topping to lifestyle."}]</t>
         </is>
       </c>
-      <c r="G2" s="8" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Bablatala, Tentultala, Kolkata 700136</t>
         </is>
       </c>
-      <c r="H2" s="8" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>Rechi Nirmaan (P) Ltd.</t>
         </is>
       </c>
-      <c r="I2" s="8" t="inlineStr">
-        <is>
-          <t>Ongoing</t>
-        </is>
-      </c>
-      <c r="J2" s="8" t="n"/>
-      <c r="K2" s="8" t="n"/>
-      <c r="L2" s="8" t="n"/>
-      <c r="M2" s="8" t="b">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="M2" t="b">
         <v>0</v>
       </c>
-      <c r="N2" s="7" t="n">
+      <c r="N2" t="n">
         <v>8</v>
       </c>
-      <c r="O2" s="11" t="n">
-        <v>25569.22970229167</v>
-      </c>
-      <c r="P2" s="11" t="n">
-        <v>46279.61171090456</v>
+      <c r="O2" s="16" t="n">
+        <v>46279.60673429242</v>
+      </c>
+      <c r="P2" s="16" t="n">
+        <v>46279.63275510486</v>
       </c>
     </row>
     <row r="3" ht="18.75" customHeight="1">
       <c r="A3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" t="n">
         <v>3</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>ANANDI APARTMENT</t>
+          <t>ANANDI VILLA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>anandi-apartment</t>
+          <t>anandi-villa</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -1118,7 +1114,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1, Niranjan Pally, Bablatala, Kolkata - 700136.</t>
+          <t>Debi Park, Bablatala, Kolkata - 700136</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1135,30 +1131,30 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O3" s="16" t="n">
-        <v>46279.60673429242</v>
+        <v>46279.60684176671</v>
       </c>
       <c r="P3" s="16" t="n">
-        <v>46279.60673429276</v>
+        <v>46279.60684176678</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>ANANDI VILLA</t>
+          <t>ANANDI PARK</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>anandi-villa</t>
+          <t>anandi-park</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1168,7 +1164,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Debi Park, Bablatala, Kolkata - 700136</t>
+          <t>Kajial Para, Rajarhat, Kolkata - 700135.</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1185,45 +1181,45 @@
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O4" s="16" t="n">
-        <v>46279.60684176671</v>
+        <v>46279.60694925111</v>
       </c>
       <c r="P4" s="16" t="n">
-        <v>46279.60684176678</v>
+        <v>46279.60694925119</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B5" t="n">
         <v>3</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ANANDI PARK</t>
+          <t>ANANDI ENCLAVE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>anandi-park</t>
+          <t>anandi-enclave</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>[{"type": "paragraph", "text": "Property details to be uploaded very soon......", "items": null}]</t>
+          <t>[{"type": "paragraph", "text": "Anandi Enclave by Rechi Construction Private Limited is a B+G+6 residential project consisting of 2 towers, located at Bablatala, Sourav Ganguly Avenue, Rajarhat, Kolkata - 700136, one of the prominent localities of Kolkata.", "items": null}, {"type": "paragraph", "text": "The project is situated in a superbly convenient and peaceful locality, close to Rajarhat Main Road.", "items": null}, {"type": "paragraph", "text": "The project is approximately 15 minutes' driving distance from the Airport, 10 minutes from Chinar Park, and 7 minutes from City Centre.", "items": null}]</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Kajial Para, Rajarhat, Kolkata - 700135.</t>
+          <t>Sourav Ganguly Avenue, Bablatala, Kolkata - 700136.</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Rechi Construction (P) Ltd.</t>
+          <t>Rechi Nirmaan (P) Ltd.</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -1235,45 +1231,45 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O5" s="16" t="n">
-        <v>46279.60694925111</v>
+        <v>46279.60703889436</v>
       </c>
       <c r="P5" s="16" t="n">
-        <v>46279.60694925119</v>
+        <v>46279.60703889441</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B6" t="n">
         <v>3</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ANANDI ENCLAVE</t>
+          <t>ANANDI RESIDENCY</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>anandi-enclave</t>
+          <t>anandi-residency</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>[{"type": "paragraph", "text": "Anandi Enclave by Rechi Construction Private Limited is a B+G+6 residential project consisting of 2 towers, located at Bablatala, Sourav Ganguly Avenue, Rajarhat, Kolkata - 700136, one of the prominent localities of Kolkata.", "items": null}, {"type": "paragraph", "text": "The project is situated in a superbly convenient and peaceful locality, close to Rajarhat Main Road.", "items": null}, {"type": "paragraph", "text": "The project is approximately 15 minutes' driving distance from the Airport, 10 minutes from Chinar Park, and 7 minutes from City Centre.", "items": null}]</t>
+          <t>[{"type": "paragraph", "text": "Details to be uploaded soon....", "items": null}]</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Sourav Ganguly Avenue, Bablatala, Kolkata - 700136.</t>
+          <t>Kajial Para, Rajarhat, Kolkata - 700135.</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Rechi Nirmaan (P) Ltd.</t>
+          <t>Rechi Construction (P) Ltd.</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -1285,40 +1281,40 @@
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O6" s="16" t="n">
-        <v>46279.60703889436</v>
+        <v>46279.60719757972</v>
       </c>
       <c r="P6" s="16" t="n">
-        <v>46279.60703889441</v>
+        <v>46279.60719757976</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7" t="n">
         <v>3</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ANANDI RESIDENCY</t>
+          <t>ANANDI VILLA (PHASE - 2)</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>anandi-residency</t>
+          <t>anandi-villa-phase-2</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>[{"type": "paragraph", "text": "Details to be uploaded soon....", "items": null}]</t>
+          <t>[{"type": "paragraph", "text": "Details to be uploaded very soon....", "items": null}]</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Kajial Para, Rajarhat, Kolkata - 700135.</t>
+          <t>Debi Park, bablatala, Kolkata - 700136.</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -1335,45 +1331,45 @@
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O7" s="16" t="n">
-        <v>46279.60719757972</v>
+        <v>46279.60733372439</v>
       </c>
       <c r="P7" s="16" t="n">
-        <v>46279.60719757976</v>
+        <v>46279.60733372443</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8" t="n">
         <v>3</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ANANDI VILLA (PHASE - 2)</t>
+          <t>SANTI BHAWAN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>anandi-villa-phase-2</t>
+          <t>santi-bhawan</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>[{"type": "paragraph", "text": "Details to be uploaded very soon....", "items": null}]</t>
+          <t>[{"type": "paragraph", "text": "SANTI BHAWAN is an Apartment ,which has 6 th floor.stand alone building wich is located 552 ,dum dum park,kol -55,It is near from josser road and vip road.Their has all morden facilitey, and comunication system.", "items": null}]</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Debi Park, bablatala, Kolkata - 700136.</t>
+          <t>552, Dum Dum Park, Kolkata 700055</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>Rechi Construction (P) Ltd.</t>
+          <t>Rechi Nirmaan (P) Ltd.</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -1385,130 +1381,130 @@
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O8" s="16" t="n">
-        <v>46279.60733372439</v>
+        <v>46279.60745506398</v>
       </c>
       <c r="P8" s="16" t="n">
-        <v>46279.60733372443</v>
+        <v>46279.60745506402</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>SANTI BHAWAN</t>
+          <t>Anandi View</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>santi-bhawan</t>
+          <t>anandi-view</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>[{"type": "paragraph", "text": "SANTI BHAWAN is an Apartment ,which has 6 th floor.stand alone building wich is located 552 ,dum dum park,kol -55,It is near from josser road and vip road.Their has all morden facilitey, and comunication system.", "items": null}]</t>
+          <t>[{"type": "paragraph", "text": "Property for sale in Rajarhat, Kolkata. This project, that is, Anandi View is a well designed project by Rechi Construction Pvt. Ltd. It is offering Under Construction units. If you are looking at Apartment, you should check out Anandi View. Available configurations include 2 BHK, 3 BHK. As per the area plan, Anandi View was launched in March 2024. Project possession is slated for June, 2025. There is 2 building in this project. Total number of flats at Anandi Views is 40.", "items": null}, {"type": "paragraph", "text": "Come home to Rechi Construction Pvt. Ltd. It offers multiple facilities such as Power Backup. There is 24x7 Security. These amenities make this property totally aspirational.", "items": null}, {"type": "paragraph", "text": "Social infrastructure like banks, schools and parks, Daily uses market surround Rajarhat area. It is also very well-connected to various parts of the city by public transport network.", "items": null}]</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>552, Dum Dum Park, Kolkata 700055</t>
+          <t>Kajial Para, Rajarhat, Kolkata - 700135</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Rechi Nirmaan (P) Ltd.</t>
+          <t>Rechi Construction Pvt. Ltd.</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>Ongoing</t>
         </is>
       </c>
       <c r="M9" t="b">
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="O9" s="16" t="n">
-        <v>46279.60745506398</v>
+        <v>46279.60774108313</v>
       </c>
       <c r="P9" s="16" t="n">
-        <v>46279.60745506402</v>
+        <v>46279.60774108317</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B10" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Anandi View</t>
+          <t>ANANDI SUNRISE</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>anandi-view</t>
+          <t>anandi-sunrise</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>[{"type": "paragraph", "text": "Property for sale in Rajarhat, Kolkata. This project, that is, Anandi View is a well designed project by Rechi Construction Pvt. Ltd. It is offering Under Construction units. If you are looking at Apartment, you should check out Anandi View. Available configurations include 2 BHK, 3 BHK. As per the area plan, Anandi View was launched in March 2024. Project possession is slated for June, 2025. There is 2 building in this project. Total number of flats at Anandi Views is 40.", "items": null}, {"type": "paragraph", "text": "Come home to Rechi Construction Pvt. Ltd. It offers multiple facilities such as Power Backup. There is 24x7 Security. These amenities make this property totally aspirational.", "items": null}, {"type": "paragraph", "text": "Social infrastructure like banks, schools and parks, Daily uses market surround Rajarhat area. It is also very well-connected to various parts of the city by public transport network.", "items": null}]</t>
+          <t>[{"type": "paragraph", "text": "Property details to be uploaded very soon......", "items": null}]</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Kajial Para, Rajarhat, Kolkata - 700135</t>
+          <t>Rajarhat, Basina, Kolkata - 700135.</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Rechi Construction Pvt. Ltd.</t>
+          <t>Rechi Construction (P) Ltd.</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Ongoing</t>
+          <t>Upcoming</t>
         </is>
       </c>
       <c r="M10" t="b">
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O10" s="16" t="n">
-        <v>46279.60774108313</v>
+        <v>46279.60786492439</v>
       </c>
       <c r="P10" s="16" t="n">
-        <v>46279.60774108317</v>
+        <v>46279.60786492443</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B11" t="n">
         <v>5</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ANANDI SUNRISE</t>
+          <t>ANANDI PALACE</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>anandi-sunrise</t>
+          <t>anandi-palace</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1518,12 +1514,12 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Rajarhat, Basina, Kolkata - 700135.</t>
+          <t>Rajarhat, Khamar, kolkata 700135.</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Rechi Construction (P) Ltd.</t>
+          <t>RECHI CONSTRUCTION PVT. LTD.</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -1535,45 +1531,45 @@
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="O11" s="16" t="n">
-        <v>46279.60786492439</v>
+        <v>46279.60798486778</v>
       </c>
       <c r="P11" s="16" t="n">
-        <v>46279.60786492443</v>
+        <v>46279.60798486781</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B12" t="n">
         <v>5</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>ANANDI PALACE</t>
+          <t>ANANDI GARDEN</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>anandi-palace</t>
+          <t>anandi-garden</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>[{"type": "paragraph", "text": "Property details to be uploaded very soon......", "items": null}]</t>
+          <t>[{"type": "paragraph", "text": "Check out this residential project for sale by Rechi Construction Pvt. Ltd. in Rajarhat, Kolkata. we offers G+4 complex as property type. The project has been developed in an area of 105 kathas . It is currently Under Progress. Available configurations include 2 BHK, 3 BHK. As per the area plan, . Altogether, there are 180 units available. There are 8 buildings in this property. all residents have easy access to some of the truly desired facilities such as Gymnasium, Power Backup. There is 24x7 Security. It is a Gated Community. Come home to GM Meena Paradise III. GM Group is a renowned developer firm.", "items": null}, {"type": "paragraph", "text": "Rajarhat is a prime area, with many attractions work and recreational options just a drive away. Airport on are few minutes away, Well connected to New Town, Nearest Metro cc2,", "items": null}]</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Rajarhat, Khamar, kolkata 700135.</t>
+          <t>Bhatenda, Near gas godwan, Rajarhat, Kolkata - 700135</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>RECHI CONSTRUCTION PVT. LTD.</t>
+          <t>Rechi Construction Pvt. Ltd.</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1585,40 +1581,40 @@
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="O12" s="16" t="n">
-        <v>46279.60798486778</v>
+        <v>46279.60811274526</v>
       </c>
       <c r="P12" s="16" t="n">
-        <v>46279.60798486781</v>
+        <v>46279.60811274531</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B13" t="n">
         <v>5</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>ANANDI GARDEN</t>
+          <t>ANANDI GREEN VIEW</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>anandi-garden</t>
+          <t>anandi-green-view</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>[{"type": "paragraph", "text": "Check out this residential project for sale by Rechi Construction Pvt. Ltd. in Rajarhat, Kolkata. we offers G+4 complex as property type. The project has been developed in an area of 105 kathas . It is currently Under Progress. Available configurations include 2 BHK, 3 BHK. As per the area plan, . Altogether, there are 180 units available. There are 8 buildings in this property. all residents have easy access to some of the truly desired facilities such as Gymnasium, Power Backup. There is 24x7 Security. It is a Gated Community. Come home to GM Meena Paradise III. GM Group is a renowned developer firm.", "items": null}, {"type": "paragraph", "text": "Rajarhat is a prime area, with many attractions work and recreational options just a drive away. Airport on are few minutes away, Well connected to New Town, Nearest Metro cc2,", "items": null}]</t>
+          <t>[{"type": "paragraph", "text": "The project is situated at the midst of tranquil surroundings of Rajarhat, and is merely few minutes from the CC2 metro staion,eco park,", "items": null}, {"type": "paragraph", "text": "G+7 buildings with 91 units above flats are being constructed in association with the top-most architects and engineers.", "items": null}, {"type": "paragraph", "text": "The project consists of 2 BHK and 3 BHK flats which are thoughtfully designed to offer maximum use of space.", "items": null}, {"type": "paragraph", "text": "The following facilities would be provided for the ultimate convenience of the residents:", "items": null}, {"type": "bullet_list", "text": null, "items": ["Automatic Lift", "AC Community Hall", "AC Gym", "Connected Roof", "Water Treatment Plant", "Fire Fighting System"]}, {"type": "paragraph", "text": "And of course, all these at a very affordable price.", "items": null}]</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Bhatenda, Near gas godwan, Rajarhat, Kolkata - 700135</t>
+          <t>Rajarhat, Kalikapur, Patharghata, Kolakata-700135</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -1635,63 +1631,63 @@
         <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="O13" s="16" t="n">
-        <v>46279.60811274526</v>
+        <v>46279.60826753888</v>
       </c>
       <c r="P13" s="16" t="n">
-        <v>46279.60811274531</v>
+        <v>46279.60826753893</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B14" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>ANANDI GREEN VIEW</t>
+          <t>ANANDI APARTMENT</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>anandi-green-view</t>
+          <t>anandi-apartment</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>[{"type": "paragraph", "text": "The project is situated at the midst of tranquil surroundings of Rajarhat, and is merely few minutes from the CC2 metro staion,eco park,", "items": null}, {"type": "paragraph", "text": "G+7 buildings with 91 units above flats are being constructed in association with the top-most architects and engineers.", "items": null}, {"type": "paragraph", "text": "The project consists of 2 BHK and 3 BHK flats which are thoughtfully designed to offer maximum use of space.", "items": null}, {"type": "paragraph", "text": "The following facilities would be provided for the ultimate convenience of the residents:", "items": null}, {"type": "bullet_list", "text": null, "items": ["Automatic Lift", "AC Community Hall", "AC Gym", "Connected Roof", "Water Treatment Plant", "Fire Fighting System"]}, {"type": "paragraph", "text": "And of course, all these at a very affordable price.", "items": null}]</t>
+          <t>[{"type": "paragraph", "text": "Property details to be uploaded very soon......", "items": null}]</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Rajarhat, Kalikapur, Patharghata, Kolakata-700135</t>
+          <t>1, Niranjan Pally, Bablatala, Kolkata - 700136.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Rechi Construction Pvt. Ltd.</t>
+          <t>Rechi Construction (P) Ltd.</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Upcoming</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="M14" t="b">
         <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="O14" s="16" t="n">
-        <v>46279.60826753888</v>
+        <v>46279.63409294162</v>
       </c>
       <c r="P14" s="16" t="n">
-        <v>46279.60826753893</v>
+        <v>46279.63409294165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Anandi Palace from upcming to ongoing
</commit_message>
<xml_diff>
--- a/migrated_backend/storage/RechiCMS.xlsx
+++ b/migrated_backend/storage/RechiCMS.xlsx
@@ -488,7 +488,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -610,7 +610,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -787,7 +787,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -938,7 +938,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="2" max="2"/>
@@ -1084,10 +1084,10 @@
         <v>8</v>
       </c>
       <c r="O2" s="16" t="n">
-        <v>46279.60673429242</v>
+        <v>46279.60673429398</v>
       </c>
       <c r="P2" s="16" t="n">
-        <v>46279.63275510486</v>
+        <v>46279.63275510417</v>
       </c>
     </row>
     <row r="3" ht="18.75" customHeight="1">
@@ -1134,10 +1134,10 @@
         <v>2</v>
       </c>
       <c r="O3" s="16" t="n">
-        <v>46279.60684176671</v>
+        <v>46279.60684177083</v>
       </c>
       <c r="P3" s="16" t="n">
-        <v>46279.60684176678</v>
+        <v>46279.60684177083</v>
       </c>
     </row>
     <row r="4">
@@ -1184,10 +1184,10 @@
         <v>3</v>
       </c>
       <c r="O4" s="16" t="n">
-        <v>46279.60694925111</v>
+        <v>46279.60694924768</v>
       </c>
       <c r="P4" s="16" t="n">
-        <v>46279.60694925119</v>
+        <v>46279.60694924768</v>
       </c>
     </row>
     <row r="5">
@@ -1234,10 +1234,10 @@
         <v>4</v>
       </c>
       <c r="O5" s="16" t="n">
-        <v>46279.60703889436</v>
+        <v>46279.60703888889</v>
       </c>
       <c r="P5" s="16" t="n">
-        <v>46279.60703889441</v>
+        <v>46279.60703888889</v>
       </c>
     </row>
     <row r="6">
@@ -1284,10 +1284,10 @@
         <v>5</v>
       </c>
       <c r="O6" s="16" t="n">
-        <v>46279.60719757972</v>
+        <v>46279.60719758102</v>
       </c>
       <c r="P6" s="16" t="n">
-        <v>46279.60719757976</v>
+        <v>46279.60719758102</v>
       </c>
     </row>
     <row r="7">
@@ -1334,10 +1334,10 @@
         <v>6</v>
       </c>
       <c r="O7" s="16" t="n">
-        <v>46279.60733372439</v>
+        <v>46279.60733372685</v>
       </c>
       <c r="P7" s="16" t="n">
-        <v>46279.60733372443</v>
+        <v>46279.60733372685</v>
       </c>
     </row>
     <row r="8">
@@ -1384,10 +1384,10 @@
         <v>7</v>
       </c>
       <c r="O8" s="16" t="n">
-        <v>46279.60745506398</v>
+        <v>46279.60745506945</v>
       </c>
       <c r="P8" s="16" t="n">
-        <v>46279.60745506402</v>
+        <v>46279.60745506945</v>
       </c>
     </row>
     <row r="9">
@@ -1434,10 +1434,10 @@
         <v>9</v>
       </c>
       <c r="O9" s="16" t="n">
-        <v>46279.60774108313</v>
+        <v>46279.60774108797</v>
       </c>
       <c r="P9" s="16" t="n">
-        <v>46279.60774108317</v>
+        <v>46279.60774108797</v>
       </c>
     </row>
     <row r="10">
@@ -1484,10 +1484,10 @@
         <v>10</v>
       </c>
       <c r="O10" s="16" t="n">
-        <v>46279.60786492439</v>
+        <v>46279.60786491898</v>
       </c>
       <c r="P10" s="16" t="n">
-        <v>46279.60786492443</v>
+        <v>46279.60786491898</v>
       </c>
     </row>
     <row r="11">
@@ -1495,7 +1495,7 @@
         <v>12</v>
       </c>
       <c r="B11" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1534,10 +1534,10 @@
         <v>11</v>
       </c>
       <c r="O11" s="16" t="n">
-        <v>46279.60798486778</v>
+        <v>46279.60798487269</v>
       </c>
       <c r="P11" s="16" t="n">
-        <v>46279.60798486781</v>
+        <v>46299.8699515737</v>
       </c>
     </row>
     <row r="12">
@@ -1584,10 +1584,10 @@
         <v>12</v>
       </c>
       <c r="O12" s="16" t="n">
-        <v>46279.60811274526</v>
+        <v>46279.60811274306</v>
       </c>
       <c r="P12" s="16" t="n">
-        <v>46279.60811274531</v>
+        <v>46279.60811274306</v>
       </c>
     </row>
     <row r="13">
@@ -1634,10 +1634,10 @@
         <v>13</v>
       </c>
       <c r="O13" s="16" t="n">
-        <v>46279.60826753888</v>
+        <v>46279.60826753472</v>
       </c>
       <c r="P13" s="16" t="n">
-        <v>46279.60826753893</v>
+        <v>46279.60826753472</v>
       </c>
     </row>
     <row r="14">
@@ -1684,10 +1684,10 @@
         <v>1</v>
       </c>
       <c r="O14" s="16" t="n">
-        <v>46279.63409294162</v>
+        <v>46279.63409293981</v>
       </c>
       <c r="P14" s="16" t="n">
-        <v>46279.63409294165</v>
+        <v>46279.63409293981</v>
       </c>
     </row>
   </sheetData>
@@ -1702,7 +1702,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
@@ -1816,7 +1816,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -1852,7 +1852,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -2002,7 +2002,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>

</xml_diff>

<commit_message>
Added Orchid view and orchid valley
</commit_message>
<xml_diff>
--- a/migrated_backend/storage/RechiCMS.xlsx
+++ b/migrated_backend/storage/RechiCMS.xlsx
@@ -488,7 +488,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -610,7 +610,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -787,7 +787,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -937,8 +937,8 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P14"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:P16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="2" max="2"/>
@@ -1537,7 +1537,7 @@
         <v>46279.60798487269</v>
       </c>
       <c r="P11" s="16" t="n">
-        <v>46299.8699515737</v>
+        <v>46299.86995157407</v>
       </c>
     </row>
     <row r="12">
@@ -1688,6 +1688,112 @@
       </c>
       <c r="P14" s="16" t="n">
         <v>46279.63409293981</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>16</v>
+      </c>
+      <c r="B15" t="n">
+        <v>5</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>ORCHID VALLEY</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>orchid-valley</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>[{"type": "paragraph", "text": "Details to be uploaded soon....", "items": null}]</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Sardar Para, Kaikhali, Kolkata- 700052</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Rechi Constructions</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Upcoming</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="M15" t="b">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>14</v>
+      </c>
+      <c r="O15" s="16" t="n">
+        <v>46308.54912688608</v>
+      </c>
+      <c r="P15" s="16" t="n">
+        <v>46308.5491268921</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>17</v>
+      </c>
+      <c r="B16" t="n">
+        <v>5</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>ORCHID VIEW</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>orchid-view</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>[{"type": "paragraph", "text": "Details to be uploaded soon....", "items": null}]</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Sourav GangulyAvenu,Bablatala, Kolkata- 700136.</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Rechi Constructions</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Upcoming</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr"/>
+      <c r="K16" t="inlineStr"/>
+      <c r="M16" t="b">
+        <v>0</v>
+      </c>
+      <c r="N16" t="n">
+        <v>15</v>
+      </c>
+      <c r="O16" s="16" t="n">
+        <v>46308.54980822415</v>
+      </c>
+      <c r="P16" s="16" t="n">
+        <v>46308.54980822426</v>
       </c>
     </row>
   </sheetData>
@@ -1702,7 +1808,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
@@ -1816,7 +1922,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -1852,7 +1958,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -2002,7 +2108,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>

</xml_diff>

<commit_message>
Added jaya apartments to the project list
</commit_message>
<xml_diff>
--- a/migrated_backend/storage/RechiCMS.xlsx
+++ b/migrated_backend/storage/RechiCMS.xlsx
@@ -937,7 +937,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P16"/>
+  <dimension ref="A1:P17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
@@ -1794,6 +1794,66 @@
       </c>
       <c r="P16" s="16" t="n">
         <v>46308.54980822426</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>18</v>
+      </c>
+      <c r="B17" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>JAYA APARTMENT</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>jaya-apartment</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>A ready-to-move residential apartment project by Rechi Construction Pvt. Ltd. in Kaikhali, Kolkata, offering thoughtfully planned 2 BHK homes with modern amenities and convenient connectivity.</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>[{"type": "paragraph", "text": "Jaya Apartment is a multi-storey residential project developed by Rechi Construction Pvt. Ltd., located in Mali Bagan, Sardar Para, Kaikhali, Kolkata. The project offers 2 BHK apartments designed to provide comfortable and practical living spaces.", "items": null}, {"type": "paragraph", "text": "The project comprises 18 residential units in a single G+4 tower, with apartment sizes ranging from approximately 897 to 1001 square feet. It was launched in October 2014, with possession scheduled for March 2017, and is listed as ready to move.", "items": null}, {"type": "paragraph", "text": "Residents can enjoy amenities including power backup, a water treatment plant, lift facilities, security, intercom connectivity, reserved parking, visitor parking, landscaped gardens, a swimming pool, a clubhouse, and indoor games facilities.", "items": null}, {"type": "paragraph", "text": "Situated near Kaikhali Main Road and Chiriamore, the project offers convenient access to Netaji Subhas Chandra Bose International Airport, nearby shopping destinations, educational institutions, and other essential services.", "items": null}]</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Sardarpara, Kaikhali Main Road, Chiriamore, Kolkata - 700052, West Bengal</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Rechi Construction Pvt. Ltd.</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>₹51.2 Lac - ₹58.8 Lac</t>
+        </is>
+      </c>
+      <c r="M17" t="b">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>0</v>
+      </c>
+      <c r="O17" s="16" t="n">
+        <v>46308.56803980537</v>
+      </c>
+      <c r="P17" s="16" t="n">
+        <v>46308.56803980558</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Modified Anandi view name
</commit_message>
<xml_diff>
--- a/migrated_backend/storage/RechiCMS.xlsx
+++ b/migrated_backend/storage/RechiCMS.xlsx
@@ -488,7 +488,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:H4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -610,7 +610,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:Q2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -787,7 +787,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:G4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -938,7 +938,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:P17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="2" max="2"/>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Anandi View</t>
+          <t>ANANDI VIEW</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1437,7 +1437,7 @@
         <v>46279.60774108797</v>
       </c>
       <c r="P9" s="16" t="n">
-        <v>46279.60774108797</v>
+        <v>46310.57251140091</v>
       </c>
     </row>
     <row r="10">
@@ -1707,7 +1707,6 @@
           <t>orchid-valley</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>[{"type": "paragraph", "text": "Details to be uploaded soon....", "items": null}]</t>
@@ -1728,8 +1727,6 @@
           <t>Upcoming</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="M15" t="b">
         <v>0</v>
       </c>
@@ -1737,10 +1734,10 @@
         <v>14</v>
       </c>
       <c r="O15" s="16" t="n">
-        <v>46308.54912688608</v>
+        <v>46308.54912688657</v>
       </c>
       <c r="P15" s="16" t="n">
-        <v>46308.5491268921</v>
+        <v>46308.54912688657</v>
       </c>
     </row>
     <row r="16">
@@ -1760,7 +1757,6 @@
           <t>orchid-view</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>[{"type": "paragraph", "text": "Details to be uploaded soon....", "items": null}]</t>
@@ -1781,8 +1777,6 @@
           <t>Upcoming</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="M16" t="b">
         <v>0</v>
       </c>
@@ -1790,10 +1784,10 @@
         <v>15</v>
       </c>
       <c r="O16" s="16" t="n">
-        <v>46308.54980822415</v>
+        <v>46308.54980822917</v>
       </c>
       <c r="P16" s="16" t="n">
-        <v>46308.54980822426</v>
+        <v>46308.54980822917</v>
       </c>
     </row>
     <row r="17">
@@ -1850,10 +1844,10 @@
         <v>0</v>
       </c>
       <c r="O17" s="16" t="n">
-        <v>46308.56803980537</v>
+        <v>46308.56803980324</v>
       </c>
       <c r="P17" s="16" t="n">
-        <v>46308.56803980558</v>
+        <v>46308.56803980324</v>
       </c>
     </row>
   </sheetData>
@@ -1868,7 +1862,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
@@ -1982,7 +1976,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -2018,7 +2012,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="15" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>
@@ -2168,7 +2162,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="3" min="1" max="1"/>
     <col width="13.57642857142857" bestFit="1" customWidth="1" style="8" min="2" max="2"/>

</xml_diff>